<commit_message>
Made a new excel file with wetland type (ANAE) data from most up-to-date wetland complex boundaries. Edited the wetland complex vege script to get rid of code I'm not using anymore.
</commit_message>
<xml_diff>
--- a/raw/flows_floods_15yrcomparison.xlsx
+++ b/raw/flows_floods_15yrcomparison.xlsx
@@ -5,28 +5,20 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unsw-my.sharepoint.com/personal/z5204897_ad_unsw_edu_au1/Documents/Desktop/Honours_UNSW/Assessment/RLE/Flows/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unsw-my.sharepoint.com/personal/z5204897_ad_unsw_edu_au1/Documents/Desktop/Honours_UNSW/Assessment/cumbung_assessment/raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="374" documentId="8_{B16CB74F-7F5A-422F-8531-F10FC2AE30B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{033666F6-8D05-4296-9F37-05D585B12830}"/>
+  <xr:revisionPtr revIDLastSave="493" documentId="8_{B16CB74F-7F5A-422F-8531-F10FC2AE30B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{73CF5C12-7E14-4C04-BAD8-5F7F46D0D93B}"/>
   <bookViews>
-    <workbookView xWindow="9960" yWindow="108" windowWidth="12924" windowHeight="13632" activeTab="2" xr2:uid="{B853E129-E620-4025-A24F-201758402292}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14016" activeTab="1" xr2:uid="{B853E129-E620-4025-A24F-201758402292}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
     <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
   </sheets>
-  <externalReferences>
-    <externalReference r:id="rId4"/>
-  </externalReferences>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Sheet2!$A$19:$E$28</definedName>
-    <definedName name="_xlchart.v1.0" hidden="1">Sheet2!$A$20:$A$28</definedName>
-    <definedName name="_xlchart.v1.1" hidden="1">Sheet2!$D$19</definedName>
-    <definedName name="_xlchart.v1.2" hidden="1">Sheet2!$D$20:$D$28</definedName>
-    <definedName name="_xlchart.v1.3" hidden="1">Sheet2!$E$19</definedName>
-    <definedName name="_xlchart.v1.4" hidden="1">Sheet2!$E$20:$E$28</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -288,6 +280,11 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FF4472C4"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -300,6 +297,667 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:autoTitleDeleted val="1"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet2!$D$19</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Flood change in last 50 years (%)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="50000"/>
+                <a:lumOff val="50000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="50000"/>
+                  <a:lumOff val="50000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:miter lim="800000"/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:dLbl>
+              <c:idx val="0"/>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="-7.6850988267992725E-18"/>
+                  <c:y val="3.5191783075017295E-2"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:dLblPos val="outEnd"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000001-0137-486F-AFAF-943D2D0B443E}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="1"/>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="-3.074039530719709E-17"/>
+                  <c:y val="3.7705241527740969E-2"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:dLblPos val="outEnd"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000003-0137-486F-AFAF-943D2D0B443E}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="3"/>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="-6.148079061439418E-17"/>
+                  <c:y val="3.770524152774106E-2"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:dLblPos val="outEnd"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000005-0137-486F-AFAF-943D2D0B443E}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1"/>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="outEnd"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+                <c15:leaderLines>
+                  <c:spPr>
+                    <a:ln w="9525">
+                      <a:solidFill>
+                        <a:schemeClr val="lt1">
+                          <a:lumMod val="50000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:round/>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                </c15:leaderLines>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>Sheet2!$A$20:$A$28</c:f>
+              <c:strCache>
+                <c:ptCount val="9"/>
+                <c:pt idx="0">
+                  <c:v>Great Cumbung</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Booligal wetlands</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Macquarie Marshes</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Chowilla Lindsay Walpolla</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Hattah Lakes</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Gwydir</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Lowbidgee</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Paroo Overflow Swamps</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>Yantabulla</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet2!$D$20:$D$28</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="9"/>
+                <c:pt idx="0">
+                  <c:v>-63</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>-52</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>-59</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>-54</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>-50</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>-58</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>-28</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>-18</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>25</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-7336-4873-A90F-1506C6E2ED84}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet2!$B$19</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Flow change in last 50 years (%)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="bg1">
+                <a:lumMod val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="bg1">
+                  <a:lumMod val="75000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:miter lim="800000"/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:dLbl>
+              <c:idx val="0"/>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="0"/>
+                  <c:y val="3.7705241527740969E-2"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:dLblPos val="outEnd"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000002-0137-486F-AFAF-943D2D0B443E}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="1"/>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="0"/>
+                  <c:y val="3.5191189297919936E-2"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:dLblPos val="outEnd"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000004-0137-486F-AFAF-943D2D0B443E}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="4"/>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="0"/>
+                  <c:y val="3.5191189297920124E-2"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:dLblPos val="outEnd"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000006-0137-486F-AFAF-943D2D0B443E}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1"/>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="outEnd"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+                <c15:leaderLines>
+                  <c:spPr>
+                    <a:ln w="9525">
+                      <a:solidFill>
+                        <a:schemeClr val="lt1">
+                          <a:lumMod val="50000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:round/>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                </c15:leaderLines>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>Sheet2!$A$20:$A$28</c:f>
+              <c:strCache>
+                <c:ptCount val="9"/>
+                <c:pt idx="0">
+                  <c:v>Great Cumbung</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Booligal wetlands</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Macquarie Marshes</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Chowilla Lindsay Walpolla</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Hattah Lakes</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Gwydir</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Lowbidgee</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Paroo Overflow Swamps</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>Yantabulla</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet2!$B$20:$B$28</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="9"/>
+                <c:pt idx="0">
+                  <c:v>-58</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>-58</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>-68</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>-47</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>-57</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>-56</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>-28</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>-27</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>15</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-7336-4873-A90F-1506C6E2ED84}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:dLblPos val="outEnd"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="1"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="315"/>
+        <c:overlap val="-40"/>
+        <c:axId val="162416592"/>
+        <c:axId val="162423664"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="162416592"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1100" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1"/>
+                </a:solidFill>
+                <a:effectLst>
+                  <a:glow rad="127000">
+                    <a:schemeClr val="bg1"/>
+                  </a:glow>
+                </a:effectLst>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="162423664"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="162423664"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:solidFill>
+              <a:schemeClr val="tx1"/>
+            </a:solidFill>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1"/>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="162416592"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="t"/>
+      <c:overlay val="1"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1100" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="en-US"/>
@@ -335,7 +993,7 @@
                   <a:schemeClr val="tx1"/>
                 </a:solidFill>
               </a:rPr>
-              <a:t>Flood frequency change over time</a:t>
+              <a:t>Flow frequency change over time</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -378,32 +1036,31 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>Sheet2!$D$19</c:f>
+              <c:f>Sheet2!$B$19</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Flood change in last 50 years (%)</c:v>
+                  <c:v>Flow change in last 50 years (%)</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:tx>
           <c:spPr>
-            <a:solidFill>
-              <a:schemeClr val="tx1">
-                <a:lumMod val="50000"/>
-                <a:lumOff val="50000"/>
-              </a:schemeClr>
-            </a:solidFill>
+            <a:noFill/>
             <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
               <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="50000"/>
-                  <a:lumOff val="50000"/>
-                </a:schemeClr>
+                <a:schemeClr val="accent1"/>
               </a:solidFill>
               <a:miter lim="800000"/>
             </a:ln>
-            <a:effectLst/>
+            <a:effectLst>
+              <a:glow rad="63500">
+                <a:schemeClr val="accent1">
+                  <a:satMod val="175000"/>
+                  <a:alpha val="25000"/>
+                </a:schemeClr>
+              </a:glow>
+            </a:effectLst>
           </c:spPr>
           <c:invertIfNegative val="0"/>
           <c:dLbls>
@@ -497,43 +1154,43 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet2!$D$20:$D$28</c:f>
+              <c:f>Sheet2!$B$20:$B$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="9"/>
                 <c:pt idx="0">
-                  <c:v>-63</c:v>
+                  <c:v>-58</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>-52</c:v>
+                  <c:v>-58</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>-59</c:v>
+                  <c:v>-68</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>-54</c:v>
+                  <c:v>-47</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>-50</c:v>
+                  <c:v>-57</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>-58</c:v>
+                  <c:v>-56</c:v>
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>-28</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>-18</c:v>
+                  <c:v>-27</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>25</c:v>
+                  <c:v>15</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-7336-4873-A90F-1506C6E2ED84}"/>
+              <c16:uniqueId val="{00000000-A311-4C55-AE8E-7A846E7B68E7}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -542,30 +1199,31 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>Sheet2!$E$19</c:f>
+              <c:f>Sheet2!$C$19</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Flood change since start of data (%)</c:v>
+                  <c:v>Flow change since start of data (%)</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:tx>
           <c:spPr>
-            <a:solidFill>
-              <a:schemeClr val="bg1">
-                <a:lumMod val="75000"/>
-              </a:schemeClr>
-            </a:solidFill>
+            <a:noFill/>
             <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
               <a:solidFill>
-                <a:schemeClr val="bg1">
-                  <a:lumMod val="85000"/>
-                </a:schemeClr>
+                <a:schemeClr val="accent2"/>
               </a:solidFill>
               <a:miter lim="800000"/>
             </a:ln>
-            <a:effectLst/>
+            <a:effectLst>
+              <a:glow rad="63500">
+                <a:schemeClr val="accent2">
+                  <a:satMod val="175000"/>
+                  <a:alpha val="25000"/>
+                </a:schemeClr>
+              </a:glow>
+            </a:effectLst>
           </c:spPr>
           <c:invertIfNegative val="0"/>
           <c:dLbls>
@@ -659,43 +1317,43 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet2!$E$20:$E$28</c:f>
+              <c:f>Sheet2!$C$20:$C$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="9"/>
                 <c:pt idx="0">
-                  <c:v>-73</c:v>
+                  <c:v>-75</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>-74</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>-59</c:v>
+                  <c:v>-68</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>-54</c:v>
+                  <c:v>-58</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>-71</c:v>
+                  <c:v>-57</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>-58</c:v>
+                  <c:v>-56</c:v>
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>-28</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>-18</c:v>
+                  <c:v>-27</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>25</c:v>
+                  <c:v>15</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-7336-4873-A90F-1506C6E2ED84}"/>
+              <c16:uniqueId val="{00000001-A311-4C55-AE8E-7A846E7B68E7}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -881,7 +1539,7 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="en-US"/>
@@ -917,7 +1575,7 @@
                   <a:schemeClr val="tx1"/>
                 </a:solidFill>
               </a:rPr>
-              <a:t>Flow frequency change over time</a:t>
+              <a:t>Flood frequency change over time</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -960,31 +1618,32 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>Sheet2!$B$19</c:f>
+              <c:f>Sheet2!$D$19</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Flow change in last 50 years (%)</c:v>
+                  <c:v>Flood change in last 50 years (%)</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:tx>
           <c:spPr>
-            <a:noFill/>
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="50000"/>
+                <a:lumOff val="50000"/>
+              </a:schemeClr>
+            </a:solidFill>
             <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
               <a:solidFill>
-                <a:schemeClr val="accent1"/>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="50000"/>
+                  <a:lumOff val="50000"/>
+                </a:schemeClr>
               </a:solidFill>
               <a:miter lim="800000"/>
             </a:ln>
-            <a:effectLst>
-              <a:glow rad="63500">
-                <a:schemeClr val="accent1">
-                  <a:satMod val="175000"/>
-                  <a:alpha val="25000"/>
-                </a:schemeClr>
-              </a:glow>
-            </a:effectLst>
+            <a:effectLst/>
           </c:spPr>
           <c:invertIfNegative val="0"/>
           <c:dLbls>
@@ -1078,43 +1737,43 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet2!$B$20:$B$28</c:f>
+              <c:f>Sheet2!$D$20:$D$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="9"/>
                 <c:pt idx="0">
+                  <c:v>-63</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>-52</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>-59</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>-54</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>-50</c:v>
+                </c:pt>
+                <c:pt idx="5">
                   <c:v>-58</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>-58</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>-68</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>-47</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>-57</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>-56</c:v>
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>-28</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>-27</c:v>
+                  <c:v>-18</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>15</c:v>
+                  <c:v>25</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-A311-4C55-AE8E-7A846E7B68E7}"/>
+              <c16:uniqueId val="{00000000-554D-4532-B375-B2286A168E4A}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1123,31 +1782,30 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>Sheet2!$C$19</c:f>
+              <c:f>Sheet2!$E$19</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Flow change since start of data (%)</c:v>
+                  <c:v>Flood change since start of data (%)</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:tx>
           <c:spPr>
-            <a:noFill/>
+            <a:solidFill>
+              <a:schemeClr val="bg1">
+                <a:lumMod val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
             <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
               <a:solidFill>
-                <a:schemeClr val="accent2"/>
+                <a:schemeClr val="bg1">
+                  <a:lumMod val="85000"/>
+                </a:schemeClr>
               </a:solidFill>
               <a:miter lim="800000"/>
             </a:ln>
-            <a:effectLst>
-              <a:glow rad="63500">
-                <a:schemeClr val="accent2">
-                  <a:satMod val="175000"/>
-                  <a:alpha val="25000"/>
-                </a:schemeClr>
-              </a:glow>
-            </a:effectLst>
+            <a:effectLst/>
           </c:spPr>
           <c:invertIfNegative val="0"/>
           <c:dLbls>
@@ -1241,43 +1899,43 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet2!$C$20:$C$28</c:f>
+              <c:f>Sheet2!$E$20:$E$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="9"/>
                 <c:pt idx="0">
-                  <c:v>-75</c:v>
+                  <c:v>-73</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>-74</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>-68</c:v>
+                  <c:v>-59</c:v>
                 </c:pt>
                 <c:pt idx="3">
+                  <c:v>-54</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>-71</c:v>
+                </c:pt>
+                <c:pt idx="5">
                   <c:v>-58</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>-57</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>-56</c:v>
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>-28</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>-27</c:v>
+                  <c:v>-18</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>15</c:v>
+                  <c:v>25</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-A311-4C55-AE8E-7A846E7B68E7}"/>
+              <c16:uniqueId val="{00000001-554D-4532-B375-B2286A168E4A}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1543,6 +2201,46 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="213">
   <cs:axisTitle>
@@ -2093,6 +2791,555 @@
 </file>
 
 <file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="213">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1">
+        <a:lumMod val="75000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" b="1" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1">
+        <a:lumMod val="75000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1">
+        <a:lumMod val="75000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1">
+        <a:lumMod val="15000"/>
+        <a:lumOff val="85000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:effectRef>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:miter lim="800000"/>
+      </a:ln>
+      <a:effectLst>
+        <a:glow rad="63500">
+          <a:schemeClr val="phClr">
+            <a:satMod val="175000"/>
+            <a:alpha val="25000"/>
+          </a:schemeClr>
+        </a:glow>
+      </a:effectLst>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:effectRef>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:miter lim="800000"/>
+      </a:ln>
+      <a:effectLst>
+        <a:glow rad="63500">
+          <a:schemeClr val="phClr">
+            <a:satMod val="175000"/>
+            <a:alpha val="25000"/>
+          </a:schemeClr>
+        </a:glow>
+      </a:effectLst>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:effectRef>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="22225" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+      <a:effectLst>
+        <a:glow rad="139700">
+          <a:schemeClr val="phClr">
+            <a:satMod val="175000"/>
+            <a:alpha val="14000"/>
+          </a:schemeClr>
+        </a:glow>
+      </a:effectLst>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:effectRef>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr">
+          <a:lumMod val="60000"/>
+          <a:lumOff val="40000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:effectLst>
+        <a:glow rad="63500">
+          <a:schemeClr val="phClr">
+            <a:satMod val="175000"/>
+            <a:alpha val="25000"/>
+          </a:schemeClr>
+        </a:glow>
+      </a:effectLst>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="4"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1">
+        <a:lumMod val="75000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="50000"/>
+          <a:lumOff val="50000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="100000">
+              <a:schemeClr val="dk1">
+                <a:lumMod val="75000"/>
+                <a:lumOff val="25000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="0">
+              <a:schemeClr val="dk1">
+                <a:lumMod val="65000"/>
+                <a:lumOff val="35000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="100000">
+              <a:schemeClr val="dk1">
+                <a:lumMod val="75000"/>
+                <a:lumOff val="25000"/>
+                <a:alpha val="25000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="0">
+              <a:schemeClr val="dk1">
+                <a:lumMod val="65000"/>
+                <a:lumOff val="35000"/>
+                <a:alpha val="25000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1">
+        <a:lumMod val="75000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1">
+        <a:lumMod val="75000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1">
+        <a:lumMod val="85000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="1" kern="1200" cap="none" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="25400" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr">
+            <a:alpha val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1">
+        <a:lumMod val="75000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1">
+          <a:lumMod val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1">
+        <a:lumMod val="75000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style3.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="213">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -2669,243 +3916,33 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="8051181" y="5488815"/>
-          <a:ext cx="7611265" cy="5139133"/>
+          <a:off x="8018583" y="5360488"/>
+          <a:ext cx="7581174" cy="5015230"/>
           <a:chOff x="548026" y="5948147"/>
           <a:chExt cx="7566660" cy="5055870"/>
         </a:xfrm>
       </xdr:grpSpPr>
-      <xdr:grpSp>
-        <xdr:nvGrpSpPr>
-          <xdr:cNvPr id="2" name="Group 1">
+      <xdr:graphicFrame macro="">
+        <xdr:nvGraphicFramePr>
+          <xdr:cNvPr id="3" name="Chart 2">
             <a:extLst>
               <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{221BFE0E-3324-4566-89BA-A77CCC2725EC}"/>
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{10B26254-1672-4AAD-B4A9-6F2633E0DDA5}"/>
               </a:ext>
             </a:extLst>
           </xdr:cNvPr>
-          <xdr:cNvGrpSpPr/>
-        </xdr:nvGrpSpPr>
-        <xdr:grpSpPr>
-          <a:xfrm>
-            <a:off x="548026" y="5948147"/>
-            <a:ext cx="7566660" cy="5055870"/>
-            <a:chOff x="418486" y="1501877"/>
-            <a:chExt cx="7566660" cy="5055870"/>
-          </a:xfrm>
-        </xdr:grpSpPr>
-        <xdr:graphicFrame macro="">
-          <xdr:nvGraphicFramePr>
-            <xdr:cNvPr id="3" name="Chart 2">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{10B26254-1672-4AAD-B4A9-6F2633E0DDA5}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvGraphicFramePr/>
-          </xdr:nvGraphicFramePr>
-          <xdr:xfrm>
-            <a:off x="418486" y="1501877"/>
-            <a:ext cx="7566660" cy="5055870"/>
-          </xdr:xfrm>
-          <a:graphic>
-            <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-              <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-            </a:graphicData>
-          </a:graphic>
-        </xdr:graphicFrame>
-        <xdr:cxnSp macro="">
-          <xdr:nvCxnSpPr>
-            <xdr:cNvPr id="14" name="Straight Connector 13">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CC8B10BB-6936-49FC-A339-BF97BCF0893D}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvCxnSpPr/>
-          </xdr:nvCxnSpPr>
-          <xdr:spPr>
-            <a:xfrm>
-              <a:off x="763003" y="4933166"/>
-              <a:ext cx="7078980" cy="0"/>
-            </a:xfrm>
-            <a:prstGeom prst="line">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:ln>
-              <a:solidFill>
-                <a:schemeClr val="bg2">
-                  <a:lumMod val="25000"/>
-                </a:schemeClr>
-              </a:solidFill>
-            </a:ln>
-            <a:effectLst/>
-          </xdr:spPr>
-          <xdr:style>
-            <a:lnRef idx="1">
-              <a:schemeClr val="accent1"/>
-            </a:lnRef>
-            <a:fillRef idx="0">
-              <a:schemeClr val="accent1"/>
-            </a:fillRef>
-            <a:effectRef idx="0">
-              <a:schemeClr val="accent1"/>
-            </a:effectRef>
-            <a:fontRef idx="minor">
-              <a:schemeClr val="tx1"/>
-            </a:fontRef>
-          </xdr:style>
-        </xdr:cxnSp>
-        <xdr:cxnSp macro="">
-          <xdr:nvCxnSpPr>
-            <xdr:cNvPr id="15" name="Straight Connector 14">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{65A0B72A-68B8-4376-85D3-EDA446D90E23}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvCxnSpPr/>
-          </xdr:nvCxnSpPr>
-          <xdr:spPr>
-            <a:xfrm>
-              <a:off x="755383" y="5119855"/>
-              <a:ext cx="7078980" cy="19050"/>
-            </a:xfrm>
-            <a:prstGeom prst="line">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:ln>
-              <a:solidFill>
-                <a:schemeClr val="bg1">
-                  <a:lumMod val="75000"/>
-                </a:schemeClr>
-              </a:solidFill>
-            </a:ln>
-          </xdr:spPr>
-          <xdr:style>
-            <a:lnRef idx="1">
-              <a:schemeClr val="accent2"/>
-            </a:lnRef>
-            <a:fillRef idx="0">
-              <a:schemeClr val="accent2"/>
-            </a:fillRef>
-            <a:effectRef idx="0">
-              <a:schemeClr val="accent2"/>
-            </a:effectRef>
-            <a:fontRef idx="minor">
-              <a:schemeClr val="tx1"/>
-            </a:fontRef>
-          </xdr:style>
-        </xdr:cxnSp>
-        <xdr:sp macro="" textlink="">
-          <xdr:nvSpPr>
-            <xdr:cNvPr id="16" name="TextBox 15">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5B085CE2-54D7-4D29-9A27-7E458488FD73}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvSpPr txBox="1"/>
-          </xdr:nvSpPr>
-          <xdr:spPr>
-            <a:xfrm>
-              <a:off x="6843763" y="4681706"/>
-              <a:ext cx="1080937" cy="264560"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-            <a:effectLst/>
-          </xdr:spPr>
-          <xdr:style>
-            <a:lnRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:lnRef>
-            <a:fillRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:fillRef>
-            <a:effectRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:effectRef>
-            <a:fontRef idx="minor">
-              <a:schemeClr val="tx1"/>
-            </a:fontRef>
-          </xdr:style>
-          <xdr:txBody>
-            <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="t">
-              <a:spAutoFit/>
-            </a:bodyPr>
-            <a:lstStyle/>
-            <a:p>
-              <a:r>
-                <a:rPr lang="en-AU" sz="1100">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                </a:rPr>
-                <a:t>Average = -39.6</a:t>
-              </a:r>
-            </a:p>
-          </xdr:txBody>
-        </xdr:sp>
-        <xdr:sp macro="" textlink="">
-          <xdr:nvSpPr>
-            <xdr:cNvPr id="17" name="TextBox 16">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{55E9F719-AEF9-4128-B6E7-6630A6914E30}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvSpPr txBox="1"/>
-          </xdr:nvSpPr>
-          <xdr:spPr>
-            <a:xfrm>
-              <a:off x="6851384" y="5108425"/>
-              <a:ext cx="1080937" cy="264560"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-          </xdr:spPr>
-          <xdr:style>
-            <a:lnRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:lnRef>
-            <a:fillRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:fillRef>
-            <a:effectRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:effectRef>
-            <a:fontRef idx="minor">
-              <a:schemeClr val="tx1"/>
-            </a:fontRef>
-          </xdr:style>
-          <xdr:txBody>
-            <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="t">
-              <a:spAutoFit/>
-            </a:bodyPr>
-            <a:lstStyle/>
-            <a:p>
-              <a:r>
-                <a:rPr lang="en-AU" sz="1100">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                </a:rPr>
-                <a:t>Average = -45.6</a:t>
-              </a:r>
-            </a:p>
-          </xdr:txBody>
-        </xdr:sp>
-      </xdr:grpSp>
+          <xdr:cNvGraphicFramePr/>
+        </xdr:nvGraphicFramePr>
+        <xdr:xfrm>
+          <a:off x="548026" y="5948147"/>
+          <a:ext cx="7566660" cy="5055870"/>
+        </xdr:xfrm>
+        <a:graphic>
+          <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+            <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          </a:graphicData>
+        </a:graphic>
+      </xdr:graphicFrame>
       <xdr:cxnSp macro="">
         <xdr:nvCxnSpPr>
           <xdr:cNvPr id="20" name="Straight Connector 19">
@@ -2919,7 +3956,7 @@
         </xdr:nvCxnSpPr>
         <xdr:spPr>
           <a:xfrm>
-            <a:off x="884923" y="7882105"/>
+            <a:off x="875684" y="7671836"/>
             <a:ext cx="7078980" cy="0"/>
           </a:xfrm>
           <a:prstGeom prst="line">
@@ -2987,179 +4024,1417 @@
     </xdr:graphicFrame>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>26</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>38</xdr:col>
+      <xdr:colOff>251460</xdr:colOff>
+      <xdr:row>57</xdr:row>
+      <xdr:rowOff>121084</xdr:rowOff>
+    </xdr:to>
+    <xdr:grpSp>
+      <xdr:nvGrpSpPr>
+        <xdr:cNvPr id="11" name="Group 10">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{30276186-0690-4954-9C21-8AA60F4B98C5}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGrpSpPr/>
+      </xdr:nvGrpSpPr>
+      <xdr:grpSpPr>
+        <a:xfrm>
+          <a:off x="15881048" y="5442857"/>
+          <a:ext cx="7581174" cy="5019656"/>
+          <a:chOff x="548026" y="5948147"/>
+          <a:chExt cx="7566660" cy="5055870"/>
+        </a:xfrm>
+      </xdr:grpSpPr>
+      <xdr:grpSp>
+        <xdr:nvGrpSpPr>
+          <xdr:cNvPr id="12" name="Group 11">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{26B34A45-F13C-4487-8207-1D60210FE958}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvGrpSpPr/>
+        </xdr:nvGrpSpPr>
+        <xdr:grpSpPr>
+          <a:xfrm>
+            <a:off x="548026" y="5948147"/>
+            <a:ext cx="7566660" cy="5055870"/>
+            <a:chOff x="418486" y="1501877"/>
+            <a:chExt cx="7566660" cy="5055870"/>
+          </a:xfrm>
+        </xdr:grpSpPr>
+        <xdr:graphicFrame macro="">
+          <xdr:nvGraphicFramePr>
+            <xdr:cNvPr id="18" name="Chart 17">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7E72D9FB-F234-489E-A8B8-D7AC7B600321}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvGraphicFramePr/>
+          </xdr:nvGraphicFramePr>
+          <xdr:xfrm>
+            <a:off x="418486" y="1501877"/>
+            <a:ext cx="7566660" cy="5055870"/>
+          </xdr:xfrm>
+          <a:graphic>
+            <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+              <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+            </a:graphicData>
+          </a:graphic>
+        </xdr:graphicFrame>
+        <xdr:cxnSp macro="">
+          <xdr:nvCxnSpPr>
+            <xdr:cNvPr id="19" name="Straight Connector 18">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D9B3F7AF-1288-4106-ACE7-C4A6773A955B}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvCxnSpPr/>
+          </xdr:nvCxnSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="763003" y="4933166"/>
+              <a:ext cx="7078980" cy="0"/>
+            </a:xfrm>
+            <a:prstGeom prst="line">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:ln>
+              <a:solidFill>
+                <a:schemeClr val="bg2">
+                  <a:lumMod val="25000"/>
+                </a:schemeClr>
+              </a:solidFill>
+            </a:ln>
+            <a:effectLst/>
+          </xdr:spPr>
+          <xdr:style>
+            <a:lnRef idx="1">
+              <a:schemeClr val="accent1"/>
+            </a:lnRef>
+            <a:fillRef idx="0">
+              <a:schemeClr val="accent1"/>
+            </a:fillRef>
+            <a:effectRef idx="0">
+              <a:schemeClr val="accent1"/>
+            </a:effectRef>
+            <a:fontRef idx="minor">
+              <a:schemeClr val="tx1"/>
+            </a:fontRef>
+          </xdr:style>
+        </xdr:cxnSp>
+        <xdr:cxnSp macro="">
+          <xdr:nvCxnSpPr>
+            <xdr:cNvPr id="23" name="Straight Connector 22">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7210386E-79E8-4403-8578-E84F799B41D6}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvCxnSpPr/>
+          </xdr:nvCxnSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="755383" y="5119855"/>
+              <a:ext cx="7078980" cy="19050"/>
+            </a:xfrm>
+            <a:prstGeom prst="line">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:ln>
+              <a:solidFill>
+                <a:schemeClr val="bg1">
+                  <a:lumMod val="75000"/>
+                </a:schemeClr>
+              </a:solidFill>
+            </a:ln>
+          </xdr:spPr>
+          <xdr:style>
+            <a:lnRef idx="1">
+              <a:schemeClr val="accent2"/>
+            </a:lnRef>
+            <a:fillRef idx="0">
+              <a:schemeClr val="accent2"/>
+            </a:fillRef>
+            <a:effectRef idx="0">
+              <a:schemeClr val="accent2"/>
+            </a:effectRef>
+            <a:fontRef idx="minor">
+              <a:schemeClr val="tx1"/>
+            </a:fontRef>
+          </xdr:style>
+        </xdr:cxnSp>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="24" name="TextBox 23">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9A8C6B87-BC1D-4B99-B364-1E20750F05F6}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr txBox="1"/>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="6843763" y="4681706"/>
+              <a:ext cx="1080937" cy="264560"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+            <a:effectLst/>
+          </xdr:spPr>
+          <xdr:style>
+            <a:lnRef idx="0">
+              <a:scrgbClr r="0" g="0" b="0"/>
+            </a:lnRef>
+            <a:fillRef idx="0">
+              <a:scrgbClr r="0" g="0" b="0"/>
+            </a:fillRef>
+            <a:effectRef idx="0">
+              <a:scrgbClr r="0" g="0" b="0"/>
+            </a:effectRef>
+            <a:fontRef idx="minor">
+              <a:schemeClr val="tx1"/>
+            </a:fontRef>
+          </xdr:style>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="t">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:r>
+                <a:rPr lang="en-AU" sz="1100">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                </a:rPr>
+                <a:t>Average = -39.6</a:t>
+              </a:r>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="25" name="TextBox 24">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1E0D4294-DC4C-4DE7-85E2-3780C76E0776}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr txBox="1"/>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="6851384" y="5108425"/>
+              <a:ext cx="1080937" cy="264560"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+          </xdr:spPr>
+          <xdr:style>
+            <a:lnRef idx="0">
+              <a:scrgbClr r="0" g="0" b="0"/>
+            </a:lnRef>
+            <a:fillRef idx="0">
+              <a:scrgbClr r="0" g="0" b="0"/>
+            </a:fillRef>
+            <a:effectRef idx="0">
+              <a:scrgbClr r="0" g="0" b="0"/>
+            </a:effectRef>
+            <a:fontRef idx="minor">
+              <a:schemeClr val="tx1"/>
+            </a:fontRef>
+          </xdr:style>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="t">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:r>
+                <a:rPr lang="en-AU" sz="1100">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                </a:rPr>
+                <a:t>Average = -45.6</a:t>
+              </a:r>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </xdr:grpSp>
+      <xdr:cxnSp macro="">
+        <xdr:nvCxnSpPr>
+          <xdr:cNvPr id="13" name="Straight Connector 12">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D2847DBE-9968-4D97-8E65-0D2581916C42}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvCxnSpPr/>
+        </xdr:nvCxnSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="884923" y="7882105"/>
+            <a:ext cx="7078980" cy="0"/>
+          </a:xfrm>
+          <a:prstGeom prst="line">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:ln>
+            <a:solidFill>
+              <a:schemeClr val="tx1"/>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:lnRef>
+          <a:fillRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="tx1"/>
+          </a:fontRef>
+        </xdr:style>
+      </xdr:cxnSp>
+    </xdr:grpSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>229220</xdr:colOff>
+      <xdr:row>51</xdr:row>
+      <xdr:rowOff>126999</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>371709</xdr:colOff>
+      <xdr:row>55</xdr:row>
+      <xdr:rowOff>61951</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="4" name="Rectangle 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E236FDD1-AE6F-4F0C-AB04-66684432A64F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8780553" y="9379856"/>
+          <a:ext cx="142489" cy="660666"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="bg1">
+            <a:lumMod val="65000"/>
+            <a:alpha val="0"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:ln>
+          <a:solidFill>
+            <a:schemeClr val="bg1">
+              <a:lumMod val="65000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="50000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="en-AU" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>538974</xdr:colOff>
+      <xdr:row>54</xdr:row>
+      <xdr:rowOff>136292</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>387195</xdr:colOff>
+      <xdr:row>55</xdr:row>
+      <xdr:rowOff>176561</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="5" name="TextBox 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9581E98A-C6BB-4826-9438-8B6767E38159}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8479498" y="9933435"/>
+          <a:ext cx="459030" cy="221697"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525" cmpd="sng">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-AU" sz="900"/>
+            <a:t>-73</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>32214</xdr:colOff>
+      <xdr:row>52</xdr:row>
+      <xdr:rowOff>142487</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>174703</xdr:colOff>
+      <xdr:row>54</xdr:row>
+      <xdr:rowOff>164619</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="27" name="Rectangle 26">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E1D913A8-69E5-4544-82B6-7FE5359104F2}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8583547" y="9576773"/>
+          <a:ext cx="142489" cy="384989"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+            <a:alpha val="0"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:ln>
+          <a:solidFill>
+            <a:schemeClr val="tx1">
+              <a:lumMod val="65000"/>
+              <a:lumOff val="35000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="50000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="en-AU" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>124521</xdr:colOff>
+      <xdr:row>55</xdr:row>
+      <xdr:rowOff>3717</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>582961</xdr:colOff>
+      <xdr:row>56</xdr:row>
+      <xdr:rowOff>43986</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="31" name="TextBox 30">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E9CC2F98-5130-4FA6-B103-554A51DC30B1}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8675854" y="9982288"/>
+          <a:ext cx="458440" cy="221698"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525" cmpd="sng">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-AU" sz="900"/>
+            <a:t>-75</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>209394</xdr:colOff>
+      <xdr:row>50</xdr:row>
+      <xdr:rowOff>68146</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>351883</xdr:colOff>
+      <xdr:row>55</xdr:row>
+      <xdr:rowOff>28946</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="32" name="Rectangle 31">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A0F0C8EE-2503-44EC-853B-55DAFC89E7F8}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9398218" y="9032852"/>
+          <a:ext cx="142489" cy="857270"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+            <a:alpha val="0"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:ln>
+          <a:solidFill>
+            <a:schemeClr val="tx1">
+              <a:lumMod val="65000"/>
+              <a:lumOff val="35000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="50000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="en-AU" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>106555</xdr:colOff>
+      <xdr:row>54</xdr:row>
+      <xdr:rowOff>156117</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>564995</xdr:colOff>
+      <xdr:row>56</xdr:row>
+      <xdr:rowOff>13630</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="33" name="TextBox 32">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{56867C46-0B30-484A-8225-ECA62DBBC363}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9295379" y="9837999"/>
+          <a:ext cx="458440" cy="216102"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525" cmpd="sng">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-AU" sz="900"/>
+            <a:t>-74</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>409498</xdr:colOff>
+      <xdr:row>51</xdr:row>
+      <xdr:rowOff>124521</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>551987</xdr:colOff>
+      <xdr:row>55</xdr:row>
+      <xdr:rowOff>27878</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="34" name="Rectangle 33">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D56C6967-4154-4F51-87D0-F803A6DCD6DD}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9598322" y="9268521"/>
+          <a:ext cx="142489" cy="620533"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="bg1">
+            <a:lumMod val="65000"/>
+            <a:alpha val="0"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:ln>
+          <a:solidFill>
+            <a:schemeClr val="bg1">
+              <a:lumMod val="65000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="50000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="en-AU" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>305419</xdr:colOff>
+      <xdr:row>54</xdr:row>
+      <xdr:rowOff>159834</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>153640</xdr:colOff>
+      <xdr:row>56</xdr:row>
+      <xdr:rowOff>17347</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="35" name="TextBox 34">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2CF4B252-7BBF-4C26-82E6-BF34246FDC6B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9494243" y="9841716"/>
+          <a:ext cx="460809" cy="216102"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525" cmpd="sng">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-AU" sz="900"/>
+            <a:t>-74</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>562516</xdr:colOff>
+      <xdr:row>50</xdr:row>
+      <xdr:rowOff>143107</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>94786</xdr:colOff>
+      <xdr:row>51</xdr:row>
+      <xdr:rowOff>114611</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="36" name="Rectangle 35">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{09890EDA-CEA5-4ECB-B358-007DEFC8C77F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="10976516" y="9107813"/>
+          <a:ext cx="144858" cy="150798"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+            <a:alpha val="0"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:ln>
+          <a:solidFill>
+            <a:schemeClr val="tx1">
+              <a:lumMod val="65000"/>
+              <a:lumOff val="35000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="50000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="en-AU" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>470209</xdr:colOff>
+      <xdr:row>51</xdr:row>
+      <xdr:rowOff>64429</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>318430</xdr:colOff>
+      <xdr:row>52</xdr:row>
+      <xdr:rowOff>104698</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="38" name="TextBox 37">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3D7F9025-4F75-4356-9251-E588DE83357F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="10884209" y="9208429"/>
+          <a:ext cx="460809" cy="219563"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525" cmpd="sng">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-AU" sz="900"/>
+            <a:t>-58</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>332678</xdr:colOff>
+      <xdr:row>51</xdr:row>
+      <xdr:rowOff>84873</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>475167</xdr:colOff>
+      <xdr:row>54</xdr:row>
+      <xdr:rowOff>61952</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="39" name="Rectangle 38">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B687DC3A-DE08-4F63-A561-9D3F040BCB3C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="11971854" y="9228873"/>
+          <a:ext cx="142489" cy="514961"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="bg1">
+            <a:lumMod val="65000"/>
+            <a:alpha val="0"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:ln>
+          <a:solidFill>
+            <a:schemeClr val="bg1">
+              <a:lumMod val="65000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="50000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="en-AU" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>237893</xdr:colOff>
+      <xdr:row>54</xdr:row>
+      <xdr:rowOff>11771</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>86114</xdr:colOff>
+      <xdr:row>55</xdr:row>
+      <xdr:rowOff>52040</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="40" name="TextBox 39">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3E0D836B-1487-40AD-A10B-6558EED614B6}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="11877069" y="9693653"/>
+          <a:ext cx="460810" cy="219563"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525" cmpd="sng">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-AU" sz="900"/>
+            <a:t>-71</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>574139</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>66053</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>42611</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>140369</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="41" name="Rectangle 40">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{61A9992C-7280-440D-8CC0-284E18B854EF}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9762963" y="5624171"/>
+          <a:ext cx="81060" cy="74316"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+            <a:alpha val="0"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:ln>
+          <a:solidFill>
+            <a:schemeClr val="tx1">
+              <a:lumMod val="65000"/>
+              <a:lumOff val="35000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="50000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="en-AU" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>402533</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>65031</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>481265</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>141391</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="42" name="Rectangle 41">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{364B9D4F-71B5-4C67-9245-B77BCC7988DF}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="11975408" y="5737419"/>
+          <a:ext cx="78732" cy="76360"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="bg1">
+            <a:lumMod val="65000"/>
+            <a:alpha val="0"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:ln>
+          <a:solidFill>
+            <a:schemeClr val="bg1">
+              <a:lumMod val="65000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="50000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="en-AU" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>592477</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>147330</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>446171</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>4620</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="43" name="TextBox 42">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D2326431-83A2-44F6-BB95-CE6C9EDEDC87}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9781301" y="5526154"/>
+          <a:ext cx="2304046" cy="215878"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525" cmpd="sng">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-AU" sz="1100"/>
+            <a:t>Flood change since start of data (%)</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>424035</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>147330</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>23</xdr:col>
+      <xdr:colOff>277729</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>4620</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="44" name="TextBox 43">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5FEE322C-4C86-4435-B2CD-59D1BA70A103}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="11996910" y="5636738"/>
+          <a:ext cx="2290089" cy="223250"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525" cmpd="sng">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-AU" sz="1100"/>
+            <a:t>Flow change since start of data (%)</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
-</file>
-
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <sheetNames>
-      <sheetName val="summary"/>
-      <sheetName val="graph"/>
-      <sheetName val="fourmileweir"/>
-      <sheetName val="corrong"/>
-      <sheetName val="booligal"/>
-      <sheetName val="bool_predCumb"/>
-      <sheetName val="bool_floods_unique"/>
-      <sheetName val="flow2SAdaily"/>
-      <sheetName val="flow2SAmonthly"/>
-      <sheetName val="renmark_dom_PS"/>
-      <sheetName val="chowilla_murrayL10"/>
-      <sheetName val="gwydir_yarra"/>
-      <sheetName val="hattah_barham"/>
-      <sheetName val="hattah_colignan"/>
-      <sheetName val="lowbid_redbank"/>
-      <sheetName val="lowbid_narran"/>
-      <sheetName val="paroo_xing"/>
-      <sheetName val="yanta_corr"/>
-      <sheetName val="yanta_turra"/>
-      <sheetName val="yanta_wyandra"/>
-      <sheetName val="mac_oxley"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1">
-        <row r="1">
-          <cell r="B1" t="str">
-            <v>Flood change in last 50 years (%)</v>
-          </cell>
-          <cell r="C1" t="str">
-            <v>Flood change since start of data (%)</v>
-          </cell>
-        </row>
-        <row r="2">
-          <cell r="A2" t="str">
-            <v>Gwydir</v>
-          </cell>
-          <cell r="B2">
-            <v>-91</v>
-          </cell>
-          <cell r="C2">
-            <v>-99</v>
-          </cell>
-        </row>
-        <row r="3">
-          <cell r="A3" t="str">
-            <v>Macquarie Marshes</v>
-          </cell>
-          <cell r="B3">
-            <v>-68</v>
-          </cell>
-          <cell r="C3">
-            <v>-78</v>
-          </cell>
-        </row>
-        <row r="4">
-          <cell r="A4" t="str">
-            <v>Great Cumbung</v>
-          </cell>
-          <cell r="B4">
-            <v>-67</v>
-          </cell>
-          <cell r="C4">
-            <v>-79</v>
-          </cell>
-        </row>
-        <row r="5">
-          <cell r="A5" t="str">
-            <v>Booligal wetlands</v>
-          </cell>
-          <cell r="B5">
-            <v>-67</v>
-          </cell>
-          <cell r="C5">
-            <v>-79</v>
-          </cell>
-        </row>
-        <row r="6">
-          <cell r="A6" t="str">
-            <v>Chowilla Lindsay Walpolla</v>
-          </cell>
-          <cell r="B6">
-            <v>-63</v>
-          </cell>
-          <cell r="C6">
-            <v>-79</v>
-          </cell>
-        </row>
-        <row r="7">
-          <cell r="A7" t="str">
-            <v>Renmark</v>
-          </cell>
-          <cell r="B7">
-            <v>-63</v>
-          </cell>
-          <cell r="C7">
-            <v>-79</v>
-          </cell>
-        </row>
-        <row r="8">
-          <cell r="A8" t="str">
-            <v>Hattah Lakes</v>
-          </cell>
-          <cell r="B8">
-            <v>-50</v>
-          </cell>
-          <cell r="C8">
-            <v>-66</v>
-          </cell>
-        </row>
-        <row r="9">
-          <cell r="A9" t="str">
-            <v>Lowbidgee</v>
-          </cell>
-          <cell r="B9">
-            <v>-49</v>
-          </cell>
-          <cell r="C9">
-            <v>-65</v>
-          </cell>
-        </row>
-        <row r="10">
-          <cell r="A10" t="str">
-            <v>Paroo Overflow Swamps</v>
-          </cell>
-          <cell r="B10">
-            <v>-27</v>
-          </cell>
-          <cell r="C10">
-            <v>-27</v>
-          </cell>
-        </row>
-        <row r="11">
-          <cell r="A11" t="str">
-            <v>Yantabulla</v>
-          </cell>
-          <cell r="B11">
-            <v>46</v>
-          </cell>
-          <cell r="C11">
-            <v>46</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="2"/>
-      <sheetData sheetId="3"/>
-      <sheetData sheetId="4"/>
-      <sheetData sheetId="5"/>
-      <sheetData sheetId="6"/>
-      <sheetData sheetId="7"/>
-      <sheetData sheetId="8"/>
-      <sheetData sheetId="9"/>
-      <sheetData sheetId="10"/>
-      <sheetData sheetId="11"/>
-      <sheetData sheetId="12"/>
-      <sheetData sheetId="13"/>
-      <sheetData sheetId="14"/>
-      <sheetData sheetId="15"/>
-      <sheetData sheetId="16"/>
-      <sheetData sheetId="17"/>
-      <sheetData sheetId="18"/>
-      <sheetData sheetId="19"/>
-      <sheetData sheetId="20"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>